<commit_message>
Soupisy 6.OG, Versorgungsgang, Sozialgebäude, Dachbereich; oprava výpočtu délek potrubí
Oprava: křivky (polylinie, oblouky, splajny) se dříve počítaly s délkou 0,
protože ezdxf Path nemá metodu length(). Uzavřené polylinie a kružnice se
nyní vyřazují jako symboly. Do každého soupisu přibyl list Poznámky.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J9BziDSBzJTVtPM6bhxvYE
</commit_message>
<xml_diff>
--- a/vystupy/1UG_soupis.xlsx
+++ b/vystupy/1UG_soupis.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Potrubí dle hladin" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Otopná tělesa" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DN popisky" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Popisy dispozice" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Poznámky" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Potrubí dle hladin" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Otopná tělesa" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DN popisky" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Popisy dispozice" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,6 +421,108 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Téma</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Poznámka</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Zdroj</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DXF výkres (jednotky mm). Hodnoty vytěženy automaticky skriptem tools/make_soupis.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Délky potrubí</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Součet délek LINE/ARC/SPLINE a otevřených polylinií na hladinách 'Heiz…'. Uzavřené polylinie, kružnice a elipsy vyřazeny (symboly těles/armatur). Jde o délku kresby, ne o ověřenou délku trubek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Kontrola V/R</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>U procesních okruhů přívod a zpátečka délkou sedí. U okruhů k otopným tělesům může být přívod nadhodnocen (symboly kreslené čarami na hladině přívodu) – ověřit ve výkresu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Výkon těles</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Párováno k nejbližšímu popisku 'P ≈ … W' (typicky 750 mm pod názvem; vzdálenost uvedena pro kontrolu). U '3x …' NENÍ ověřeno, zda výkon platí na kus, nebo celkem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Označení těles</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Význam čísel (např. 42/900/100 = články/výška/hloubka?) není ověřen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DN popisky</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pouze textové popisky s polohou; přiřazení ke konkrétnímu úseku potrubí nebylo provedeno.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -472,7 +575,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>722</v>
+        <v>601</v>
       </c>
       <c r="E2" t="n">
         <v>1547.1</v>
@@ -493,7 +596,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>655</v>
+        <v>596</v>
       </c>
       <c r="E3" t="n">
         <v>1525.1</v>
@@ -514,7 +617,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>399</v>
+        <v>375</v>
       </c>
       <c r="E4" t="n">
         <v>1124.5</v>
@@ -535,7 +638,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E5" t="n">
         <v>48.3</v>
@@ -556,7 +659,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>570</v>
+        <v>489</v>
       </c>
       <c r="E6" t="n">
         <v>1291.1</v>
@@ -577,7 +680,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E7" t="n">
         <v>48.6</v>
@@ -598,7 +701,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E8" t="n">
         <v>144.9</v>
@@ -619,7 +722,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>233</v>
+        <v>215</v>
       </c>
       <c r="E9" t="n">
         <v>515.4</v>
@@ -640,7 +743,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E10" t="n">
         <v>136.4</v>
@@ -661,7 +764,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>242</v>
+        <v>221</v>
       </c>
       <c r="E11" t="n">
         <v>505.3</v>
@@ -679,7 +782,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E12" t="n">
         <v>15.2</v>
@@ -690,7 +793,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1587,7 +1690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4449,7 +4552,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>